<commit_message>
feat(v1): M1 ledger core - chart of accounts, period states, PostingService, journals, general ledger, trial balance
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -33,12 +33,17 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -68,9 +73,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -78,6 +83,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -517,10 +525,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>account table + AccountService + /accounts API + default UK chart (UK_SMALL_COMPANY v1). migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: tests/api/ledger.test.ts (chart), tests/db/ledger.test.ts (account guards), packages/contracts/src/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -544,7 +556,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -577,7 +589,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -606,7 +618,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -635,7 +647,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -664,7 +676,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -693,7 +705,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -722,7 +734,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -751,7 +763,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -780,7 +792,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -809,7 +821,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -838,7 +850,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -873,11 +885,19 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>POST /journals (manual and opening-balance sources), GET /journals[/id], POST /journals/{id}/reverse; all through the PostingService. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Posting only: no draft or approval step for manual journals (open decision 5 in v1-plan.md)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -902,10 +922,14 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>GET /ledger (general ledger per account, running balance, keyset paging recomputed per page). Tests: tests/platform/posting-service.test.ts (one page equals paged), tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
@@ -931,10 +955,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>GET /reports/trial-balance (as at a date or a period with movement; journal lines only; balanced flag; suspense warning; drill-down parameters). Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts (independent SQL check)</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -958,7 +986,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -987,7 +1015,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1016,7 +1044,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1045,17 +1073,21 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>V0: accounting_period table with OPEN/CLOSED/LOCKED enum, no-overlap constraint, create/list API. No transition rules, no enforcement on postings.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
+          <t>OPEN&lt;-&gt;CLOSED-&gt;LOCKED-&gt;CLOSED with database-enforced graph, period:manage / period:lock, mandatory reasons, audit before/after, events, concurrency-safe. Tests: tests/platform/posting-service.test.ts (period controls), tests/db/ledger.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Close controls beyond 'ledger balances' are added by M2-M5 as their data exists (see MAN-ACC-08)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1078,12 +1110,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>PostingService -&gt; journal -&gt; journal_line -&gt; ledger exists with MANUAL, OPENING_BALANCE and REVERSAL sources. No source-document transaction services yet (M2+). Tests: tests/platform/posting-service.test.ts</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>M1 delivers PostingService + journals + ledger with manual and reversal sources; each later milestone adds a transaction service</t>
@@ -1111,12 +1147,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Trial balance and general ledger aggregate journal_line only (architecture: no report reads source tables). P&amp;L and balance sheet are M5. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Trial balance in M1; statements in M5, both from journal lines only</t>
@@ -1146,10 +1186,14 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>account.code (unique per company, 1-20 chars). migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1175,10 +1219,14 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>account.name. migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1204,10 +1252,14 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>account.type (ASSET/LIABILITY/EQUITY/INCOME/EXPENSE). migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1233,10 +1285,14 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>account.subtype (registry constrained to the type). migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1262,10 +1318,14 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>account.is_control + control_kind (receivables, payables, VAT, bank, cash, suspense, retained earnings); manual journals cannot post to control accounts. migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1291,10 +1351,14 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>account.tax_treatment (account level). migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Account-level treatment in M1; VAT codes on lines arrive with the VAT foundation (M2)</t>
@@ -1324,10 +1388,14 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>account.reporting_mapping from a versioned report-line registry, checked against the type. migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1353,10 +1421,14 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>account.active_from / active_to enforced on every posting date; deactivation cannot precede the last posting. migration 20260106000000_v1_ledger_core; packages/accounting; apps/api/src/ledger; ADR-44..48. Tests: packages/contracts/src/ledger.test.ts, tests/api/ledger.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1382,13 +1454,17 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Single writer enforced three ways: architecture test (only packages/accounting/src/posting.ts writes journal/journal_line/ledger_sequence; only it sets app.posting; platform/AI/worker cannot import the package), database guard (insert refused without the transaction flag), privileges. Tests: tests/unit/architecture.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Enforced by an architecture test, a database guard (transaction flag) and privileges</t>
+          <t>Honest limit: the flag is application-asserted (same trust boundary as tenant context)</t>
         </is>
       </c>
     </row>
@@ -1415,10 +1491,14 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Application check + deferred constraint trigger at commit (header agrees with lines, contiguous numbering, reversal mirrors original). Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1444,10 +1524,14 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Accounts must exist in the company (composite FK), be active on the journal date, and not be control accounts for manual sources. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1473,10 +1557,14 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Period must exist, contain the date and be OPEN; period row locked FOR SHARE so a concurrent close cannot race. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts (race test), tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1500,7 +1588,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1533,12 +1621,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Currency validated: journals are in the company base currency and amounts respect its minor units (application + database). Foreign-currency documents, FX rates and revaluation are NOT supported (open decision 1). Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Base currency of the company only; foreign-currency postings and FX revaluation are not in V1 scope until a decision is recorded</t>
@@ -1568,10 +1660,14 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Registered source type required; REVERSAL must name the reversed journal; other sources require a source id; idempotency key per company with content hash. Tests: tests/platform/posting-service.test.ts, packages/contracts/src/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1597,10 +1693,14 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Source-specific permission evaluated for the journal's company through the central authoriser; AI actors refused; system actors limited to system sources. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts (roles x posting), tests/api/permissions.test.ts</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1624,7 +1724,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1653,7 +1753,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1682,7 +1782,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1711,7 +1811,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1740,7 +1840,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1773,7 +1873,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1802,7 +1902,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1835,7 +1935,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1864,7 +1964,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1893,7 +1993,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1922,7 +2022,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1951,7 +2051,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -1980,7 +2080,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2009,7 +2109,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2038,7 +2138,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2067,7 +2167,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2096,7 +2196,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2129,7 +2229,7 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2158,7 +2258,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2191,12 +2291,16 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Report -&gt; account -&gt; journal -&gt; source reference works (trial balance rows carry drill-down parameters; ledger lines carry journal and source). Source transaction and document links arrive with each source module. Tests: tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Report -&gt; account -&gt; journal in M1; source transaction and document links arrive with each source module</t>
@@ -2226,10 +2330,14 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Closed and locked periods refuse postings (service + database); lock needs period:lock. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2253,7 +2361,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2282,12 +2390,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr"/>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Trial balance warns about a non-zero suspense balance (account with control kind SUSPENSE). Dashboard alert is M5. Tests: tests/platform/posting-service.test.ts</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>Trial balance warning in M1; dashboard alert in M5</t>
@@ -2315,7 +2427,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2344,7 +2456,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2373,14 +2485,14 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>V0 audit framework (append-only, before/after, reason, source workflow). Ledger actions are not yet audited.</t>
+          <t>journal.posted/reversed, account.created/updated/chart_initialised and period.closed/reopened/locked/unlocked are audited in the business transaction (before/after, reason, actor, source workflow where relevant). Source modules add their own events in M2+. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -2406,12 +2518,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr"/>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Positive, negative, reversal and period-lock tests exist for every M1 posting rule; the VAT test arrives with the VAT validator (M2). Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
           <t>Applied per rule as each milestone adds rules; the matrix lists the rule set tested</t>
@@ -2441,10 +2557,14 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Single writer enforced three ways: architecture test (only packages/accounting/src/posting.ts writes journal/journal_line/ledger_sequence; only it sets app.posting; platform/AI/worker cannot import the package), database guard (insert refused without the transaction flag), privileges. Tests: tests/unit/architecture.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
           <t>Same as V1-POST-01</t>
@@ -2474,10 +2594,14 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>No UPDATE/DELETE/TRUNCATE privilege for the runtime role and append-only triggers (the table owner is refused too). Tests: tests/db/ledger.test.ts, tests/db/privileges.test.ts</t>
+        </is>
+      </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
           <t>Privileges, triggers, tests</t>
@@ -2507,10 +2631,14 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Reversal journals: linked both ways, mirror enforced per account at commit, at most once, a reversal cannot be reversed, dated on/after the original, in an open period. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts, tests/api/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
@@ -2536,10 +2664,14 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Application validation and a deferred database check at commit. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
           <t>Application and deferred database check</t>
@@ -2569,10 +2701,14 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>journal: source_type/source_id/source_reference, actor_type + posted_by_user_id, posted_at, correlation id, idempotency key; audit event and transaction.posted outbox event in the same transaction. Tests: tests/platform/posting-service.test.ts</t>
+        </is>
+      </c>
       <c r="G70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
@@ -2596,12 +2732,16 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Journal -&gt; source via source_type/source_id/source_reference (done); source transaction -&gt; journal is delivered per source module (M2+).</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
           <t>Journal -&gt; source in M1 (source_type/source_id); source -&gt; journal per module</t>
@@ -2629,7 +2769,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2662,12 +2802,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
           <t>Same as V1-MOD-19</t>
@@ -2695,12 +2839,16 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Report mappings are a versioned registry (REPORT_MAPPING_VERSION = 1, returned with every account) but not yet effective-dated in the database; VAT rates are M2.</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
           <t>Reporting mappings versioned in M1; VAT rates effective-dated in M2</t>
@@ -2730,10 +2878,14 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>PostingService refuses AI actors (ai_cannot_post); no journal source lists AI; architecture test forbids platform, the AI module and the worker from importing the accounting package. Tests: tests/platform/posting-service.test.ts, packages/contracts/src/ledger.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
           <t>PostingService refuses AI actors; architecture test keeps the AI module away from the posting code</t>
@@ -2761,7 +2913,7 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2790,12 +2942,16 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2.</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>TransactionPosted in M1; BankImported M4; InvoiceCreated M2</t>
@@ -2823,7 +2979,7 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
@@ -2873,7 +3029,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -2883,7 +3039,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -2893,7 +3049,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -2953,7 +3109,7 @@
         <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
docs(v1): M1 acceptance package and matrix regenerated against the verified commit
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -3208,7 +3208,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fae5270</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3216,7 +3220,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37923766068</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">

</xml_diff>

<commit_message>
docs+test(privacy): DEC-013 investigation of session/challenge IP and user agent (unresolved), characterisation tests, legal schedule correction
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -6305,9 +6305,9 @@
           <t>Privacy track (parallel to V1)</t>
         </is>
       </c>
-      <c r="E114" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -6330,8 +6330,16 @@
           <t>Any deletion job (S4(b) is frozen)</t>
         </is>
       </c>
-      <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Investigation delivered: docs/legal/device-metadata-investigation.md (7 collection points traced, 6 findings F-1..F-6, options A-F proposed and NOT enabled, review checklist); 10 characterisation tests in tests/api/device-metadata.test.ts; legal schedule corrected (raw IPs in Redis rate-limit keys). The finding is UNRESOLVED: no policy, deletion or lawful basis is approved; deletion stays frozen (S4(b)).</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>Never mark resolved without the recorded privacy review</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K114"/>
@@ -6806,7 +6814,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>INVESTIGATION IN PROGRESS - never marked resolved without review</t>
+          <t>INVESTIGATION DELIVERED - finding UNRESOLVED, awaiting privacy review (never resolved without it)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -6883,7 +6891,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -6893,7 +6901,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
V1-M2: acceptance package and matrix regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -3778,7 +3778,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>journal.posted/reversed, account.created/updated/chart_initialised and period.closed/reopened/locked/unlocked are audited in the business transaction (before/after, reason, actor, source workflow where relevant). Source modules add their own events in M2+. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
+          <t>journal.posted/reversed, account.created/updated/chart_initialised and period.closed/reopened/locked/unlocked are audited in the business transaction (before/after, reason, actor, source workflow where relevant). M2 adds ledger.request_created/approved/rejected/cancelled and ledger.policy_changed (before/after, reason). Source modules add their own events in M5+. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
@@ -4578,9 +4578,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -4603,7 +4603,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Permission `ledger:opening-balance` (COMPANY scope) is required to request an opening balance; owner/admin/partner hold it, manager/accountant/bookkeeper/reviewer/client viewer do not (migration 20260107000000 + role sync). `journal:post` alone no longer suffices; `POST /journals` refuses OPENING_BALANCE. Tests: tests/api/ledger-controls.test.ts (permission matrix over 8 roles for all four new permissions, 22 cases), tests/api/permissions.test.ts (4 new probes x 8 roles), packages/contracts/src/ledger.test.ts</t>
+        </is>
+      </c>
       <c r="K79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
@@ -4627,9 +4631,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4652,7 +4656,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>CONTROL_ADJUSTMENT request needs `ledger:control-adjustment` (accountant, owner/admin/partner), a reason of at least 20 characters (service + database check), at least one evidence document that exists, belongs to the company and is readable by the requester (restricted documents indistinguishable from missing), and must touch a control account. The journal records request, requester and approver and the evidence is linked journal -&gt; document in the evidence graph; MANUAL journals still refused on control accounts. Tests: tests/api/ledger-controls.test.ts (validation, control-account adjustment, evidence graph), tests/platform/posting-service.test.ts</t>
+        </is>
+      </c>
       <c r="K80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
@@ -4676,9 +4684,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -4701,7 +4709,11 @@
           <t>Per-account rules; delegation; multi-step chains</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Per-company `ledger_policy` (ALWAYS default / ABOVE_THRESHOLD with strictly-greater materiality threshold, expiry 1-90 days; no NEVER mode - database check). Above the threshold a different person holding `ledger:approve` must approve; requester can never approve (service + database, tested against the table owner path). Below-threshold direct posting only when configured, recorded as self-approved; reject (reason required), cancel (requester only) and expiry leave the ledger untouched. Policy changes need `ledger:policy` + reason and are audited before/after. Tests: tests/api/ledger-controls.test.ts (policy, threshold boundary 1000.00 / 1000.01, concurrency), tests/db/ledger-controls.test.ts (13), tests/platform/ledger-requests.test.ts (5)</t>
+        </is>
+      </c>
       <c r="K81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
@@ -4725,9 +4737,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -4750,7 +4762,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Pending requests live in `journal_request` and are never read by trial balance / general ledger (asserted). An approved request produces exactly one journal (unique `journal.request_id`; idempotency key `request:&lt;id&gt;`; concurrent approvals and approve/reject/cancel races end with one outcome). Posted journals stay immutable and are corrected by reversal (tested); AI actors cannot request, approve or post (service + PostingService). Request content is immutable and decided requests final (trigger); no delete/truncate for runtime role or owner. Tests: tests/api/ledger-controls.test.ts, tests/db/ledger-controls.test.ts, tests/platform/ledger-requests.test.ts, tests/db/privileges.test.ts, tests/unit/architecture.test.ts (single writer of journal_request/ledger_policy)</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
@@ -4774,9 +4790,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -4799,7 +4815,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>The first-day-of-first-period rule is kept (validated at request creation and again at posting) together with the dedicated permission and the approval policy; a request dated elsewhere is refused with `opening_balance_date_invalid`. Tests: tests/api/ledger-controls.test.ts (validation), tests/platform/posting-service.test.ts</t>
+        </is>
+      </c>
       <c r="K83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
@@ -6470,7 +6490,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SPECIFIED - ready to start</t>
+          <t>IMPLEMENTED - submitted for acceptance (see v1-m2-acceptance.md for the commit, CI run and results)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -6497,7 +6517,7 @@
         <v>5</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -6881,7 +6901,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -6901,7 +6921,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -6942,7 +6962,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>fae5270</t>
+          <t>d98e3ed</t>
         </is>
       </c>
     </row>
@@ -6954,7 +6974,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37923766068</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/37933029493</t>
         </is>
       </c>
     </row>
@@ -6981,7 +7001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7008,6 +7028,13 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>v2.1 (2026-10-09): M2 ledger controls implemented. V1-CTL-07..11 -&gt; Implemented with evidence; V1-CTL-06 evidence extended. No rows added or removed; M3+ unchanged and still gated. Not accepted until the product owner says so.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record DEC-015..018 (M2 accepted; M3 rate source, rounding, revaluation); complete the M3 specification; matrix v2.2 (documentation only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -4865,7 +4865,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -4953,21 +4953,25 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Open decision: rate source</t>
+          <t>DEC-016</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Rate table with (from, to, date, rate, source, retrieved_at, verified); manual entry audited; a documented lookup rule (transaction date, else last earlier rate within N days, else refuse); an unverified rate is flagged and can be blocked by policy; a rate-source adapter port exists with a fake for tests; no live source is enabled without a recorded decision.</t>
+          <t>`exchange_rate` table (kind DAILY|PERIOD, rate to 8 dp, publisher, series, URL, retrieved_at, source_kind MANUAL|IMPORT, verification status, supersedes); manual entry needs source text and date and is audited; rows are immutable (corrections supersede); lookup = transaction date, else latest earlier DAILY rate within 7 days, else `exchange_rate_not_found`, never a future rate; CSV importer + `ExchangeRateSource` port with a fake; UNVERIFIED rates flagged and blockable by `ledger_policy.fx_block_unverified_rates`; live HTTP adapters NOT included (gate).</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
-      <c r="K86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Decision DEC-016 applied.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5012,7 +5016,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
@@ -5056,12 +5060,12 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>For every journal sum(debit)=sum(credit) in functional currency; a conversion that does not round cleanly produces an explicit rounding line to a system rounding account, capped by a tolerance; tests with awkward rates.</t>
+          <t>For every journal sum(debit)=sum(credit) in functional currency; unbalanced converted lines get one visible FX-rounding line on the system account `FX_ROUNDING`, permitted difference one minor unit per line, else `rounding_tolerance_exceeded`; tests for within/beyond tolerance.</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
@@ -5100,21 +5104,25 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Open decision: rounding policy</t>
+          <t>DEC-017</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>The policy is written (precision, mode, level), implemented in one function and covered by property tests (conversion then reverse conversion within tolerance; totals independent of line order).</t>
+          <t>Rate stored to 8 dp unrounded; functional amount rounded per line, half-up, to the functional currency's minor units by one function with property tests (reverse conversion within tolerance; totals independent of line order; half-up boundary); VAT rounding left to M4.</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
-      <c r="K89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Decision DEC-017 applied.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5154,18 +5162,18 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Settling a foreign invoice at a different rate posts the difference to realised gain/loss accounts exactly once; partial settlements prorate; tested with several rates.</t>
+          <t>`FxService.settle` posts the difference between the functional value carried and the value at the settlement rate to `FX_REALISED` exactly once; partial settlements prorate; tested with several rates (receipts/payments in M5/M6 call it).</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>Engine in M3; used by receipts and payments in M5/M6</t>
+          <t>Engine in M3; used by receipts and payments in M5/M6 Decision DEC-018 applied.</t>
         </is>
       </c>
     </row>
@@ -5202,21 +5210,25 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>V1-FX-05, open decision: revaluation policy</t>
+          <t>V1-FX-05, DEC-018</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Revaluation at period end posts unrealised gain/loss journals for foreign-currency receivables, payables and bank, and reverses on the first day of the next period; idempotent per period; blocked in locked periods; reconciles to the sub-ledger.</t>
+          <t>Explicit, previewed `revalue` action (`period:manage`) per period revalues foreign-currency monetary accounts at the period-end rate to `FX_UNREALISED`; auto-reversal dated the first day of the next period (immediately or by sweeper); idempotent per period via `fx_revaluation_run`; refused in locked periods; close needs acknowledgement if a balance is unrevalued; non-monetary items untouched.</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
-      <c r="K91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Decision DEC-018 applied.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5261,7 +5273,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting; forward contracts; intercompany eliminations</t>
+          <t>Live rate adapters (gated); hedge accounting; forward contracts; net investments; intercompany eliminations</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
@@ -6490,7 +6502,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>IMPLEMENTED - submitted for acceptance (see v1-m2-acceptance.md for the commit, CI run and results)</t>
+          <t>ACCEPTED (code baseline d98e3ed; DEC-015)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -6533,7 +6545,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SPECIFIED - open decisions block the start (exchange-rate source, rounding policy)</t>
+          <t>SPECIFIED - decisions recorded (DEC-016..018); ready to start; live rate adapters gated</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -6543,17 +6555,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>M1 accepted; M2 not required; Decision: exchange-rate source and revaluation policy (v1-plan.md section 4)</t>
+          <t>M1 accepted; M2 accepted (DEC-015); Decisions recorded: rate source and window (DEC-016), rounding (DEC-017), revaluation and realised FX (DEC-018)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Section 4 of v1-plan.md</t>
+          <t>Section 5 of v1-plan.md (5.3)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hedge accounting, forward contracts, multi-currency bank feeds (M7 handles statements in account currency only), intercompany eliminations</t>
+          <t>Live HTTP rate adapters (network, publisher terms of use and format verification), hedge accounting, forward contracts, net investments and translation of foreign operations, intercompany eliminations, multi-currency bank statements beyond the account currency (M7), VAT-specific rate rules (M4)</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -6986,7 +6998,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7035,6 +7047,13 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>v2.2 (2026-10-12, DEC-015..018): M2 ACCEPTED (code baseline d98e3ed). M3 decisions recorded (rate source and window, rounding, revaluation/realised FX); M3 specification completed in v1-plan.md section 5 and ready to start. No rows added or removed. M4 remains gated by verification of tax rules from official sources.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M3: acceptance package and matrix regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -7010,7 +7010,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>c8fd8c0</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38265470095</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V1-M4b: acceptance package; matrix regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>M4a VERIFIED (code baseline 206b14d; v1-m4a-acceptance.md); M4b IMPLEMENTED - see v1-m4b-acceptance.md. Every VAT rule is usable only after verification by the firm's holder of tax:rule-verify</t>
+          <t>M4a VERIFIED (206b14d; v1-m4a-acceptance.md); M4b VERIFIED (6fb1938; v1-m4b-acceptance.md). VAT rules usable only after verification by the firm's holder of tax:rule-verify</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>6fb1938</t>
         </is>
       </c>
     </row>
@@ -7104,7 +7104,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38311897860</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V1-M5a: acceptance package; matrix v2.6 regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -704,9 +704,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -729,8 +729,16 @@
           <t>Recurring invoices, quotes, online payment</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Invoices: DRAFT (no number, no ledger effect; revisioned lines) -&gt; APPROVED (numbered without gaps from a locked sequence the database checks; customer snapshot; amounts recomputed with verified VAT rates; posted as SALES_INVOICE Dr receivables / Cr revenue / Cr output VAT; journal and document linked both ways; immutable) or DISCARDED; attachments through the evidence graph; drafts from ACCEPTED AI proposals, approval by people only; positive, negative, VAT (standard, zero, exempt; exclusive, inclusive), period-lock and correction-by-credit-note tests. 'Paid' is reached by credit notes now; by receipts in M5b. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>M5a delivered; receipts (paid by payment) are M5b (DEC-026).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -802,9 +810,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -827,7 +835,11 @@
           <t>Refund automation</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>A sales credit note references one approved invoice of the same customer and currency (database rule), uses only the invoice's VAT codes at the invoice's rate versions (DEC-029), cannot exceed the invoice outstanding (service and database), is allocated to its invoice in the same transaction and is traceable from both documents. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1543,7 +1555,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>PostingService -&gt; journal -&gt; journal_line -&gt; ledger exists with MANUAL, OPENING_BALANCE and REVERSAL sources. No source-document transaction services yet (M2+). Tests: tests/platform/posting-service.test.ts</t>
+          <t>PostingService -&gt; journal -&gt; journal_line -&gt; ledger exists with MANUAL, OPENING_BALANCE and REVERSAL sources. No source-document transaction services yet (M2+). Tests: tests/platform/posting-service.test.ts M5a: Sales documents post only through the PostingService (SALES_INVOICE, SALES_CREDIT_NOTE, SALES_ALLOCATION_FX) and link to their journals both ways; architecture test: one writer of the sales tables, which never writes journals.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2494,9 +2506,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2519,7 +2531,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>An approved invoice posts exactly Dr trade receivables (gross) / Cr revenue (net per line) / Cr output VAT (per VAT-coded line), with standard, zero-rated and exempt lines and VAT-inclusive entry, hand-calculated. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
       <c r="K39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2690,9 +2706,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2715,7 +2731,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Sales: a credit note mirrors the credited lines and VAT, linked both ways (credit note -&gt; invoice; invoice lists its credit notes) and allocated. Purchases (debit notes) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Sales credit notes M2; purchase (debit) notes M3. The reversal primitive and source linkage ship in M1</t>
@@ -3468,7 +3488,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Report -&gt; account -&gt; journal -&gt; source reference works (trial balance rows carry drill-down parameters; ledger lines carry journal and source). Source transaction and document links arrive with each source module. Tests: tests/api/ledger.test.ts</t>
+          <t>Report -&gt; account -&gt; journal -&gt; source reference works (trial balance rows carry drill-down parameters; ledger lines carry journal and source). Source transaction and document links arrive with each source module. Tests: tests/api/ledger.test.ts M5a: Journal -&gt; sales document drill path exists (source_id) and document -&gt; journal (journal_id); report drill-down UI is M8/M9.</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3551,9 +3571,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3576,7 +3596,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Sales invoices: before approval, another approved invoice of the same customer with the same date, currency and total, or the same customer reference, refuses approval unless a reason is given (stored on the document and audited). Supplier bills (supplier's own number) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
       <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
@@ -3706,9 +3730,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3731,7 +3755,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Closing a period is refused while draft sales documents are dated in it unless acknowledged (acknowledgeDraftDocuments, recorded on the audit event); drafts are listed by status. An age threshold and alerting (dashboard) are M8. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+        </is>
+      </c>
       <c r="K63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3782,7 +3810,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>journal.posted/reversed, account.created/updated/chart_initialised and period.closed/reopened/locked/unlocked are audited in the business transaction (before/after, reason, actor, source workflow where relevant). M2 adds ledger.request_created/approved/rejected/cancelled and ledger.policy_changed (before/after, reason). Source modules add their own events in M5+. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
+          <t>journal.posted/reversed, account.created/updated/chart_initialised and period.closed/reopened/locked/unlocked are audited in the business transaction (before/after, reason, actor, source workflow where relevant). M2 adds ledger.request_created/approved/rejected/cancelled and ledger.policy_changed (before/after, reason). Source modules add their own events in M5+. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts M5a: Sales documents audit created, updated, discarded, approved (with override reasons) and allocation events.</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
@@ -4169,7 +4197,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Journal -&gt; source via source_type/source_id/source_reference (done); source transaction -&gt; journal is delivered per source module (M2+).</t>
+          <t>Journal -&gt; source via source_type/source_id/source_reference (done); source transaction -&gt; journal is delivered per source module (M2+). M5a: Sales invoices, credit notes and allocations link to their journals and back (journal source_id; document journal_id; allocation fx_journal_id), proven by database rules.</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -4279,7 +4307,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts</t>
+          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts M5a: Close control for draft sales documents dated in the period (acknowledgement recorded); unreconciled bank items follow in M7.</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4499,7 +4527,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2.</t>
+          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2. M5a: InvoiceCreated (`invoice.created`) and `credit_note.created` are published through the outbox on approval (tests/platform/sales.test.ts); BankImported is M7.</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -5200,7 +5228,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts</t>
+          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts M5a: Exercised end to end for credit-note allocations (M5a): carried amounts released by `releaseShare` (full remainder or prorated), difference posted as SALES_ALLOCATION_FX to the realised-FX account with receivables lines marked adjusts_currency; hand-calculated gain 20.00 and full-settlement 16.67 cases. Receipts and payments (M5b/M6) still to come.</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -5583,7 +5611,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Output VAT (sales codes) and input VAT (purchase codes) on journal lines, with visible VAT lines on the configured accounts. Invoices and bills are documents (M5/M6), so 'on invoices/bills' is not yet possible. Tests: tests/platform/vat.test.ts, tests/api/vat.test.ts</t>
+          <t>Output VAT (sales codes) and input VAT (purchase codes) on journal lines, with visible VAT lines on the configured accounts. Invoices and bills are documents (M5/M6), so 'on invoices/bills' is not yet possible. Tests: tests/platform/vat.test.ts, tests/api/vat.test.ts M5a: Sales invoices carry output VAT per line with the verified version at the document's tax point (M5a); purchase bills are M6.</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
@@ -5636,7 +5664,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>A credit note entered as a debit on a sales code reduces output VAT (tested); linkage to the original supply needs documents (M5/M6).</t>
+          <t>A credit note entered as a debit on a sales code reduces output VAT (tested); linkage to the original supply needs documents (M5/M6). M5a: Sales credit notes adjust VAT at the rate version the invoice used, reported at the credit note's tax point (vat_rate_point proven by the database; workpaper test); purchase debit notes are M6. Rule UNVERIFIED (DEC-029).</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr"/>
@@ -5742,7 +5770,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>Explicit tax point per journal (defaults to the journal date) selects the rate version and the return period (stagger function tested). Determining it from supply/invoice/payment dates is a document matter (M5/M6). Tests: tests/platform/vat.test.ts, tests/unit/vat-math.test.ts</t>
+          <t>Explicit tax point per journal (defaults to the journal date) selects the rate version and the return period (stagger function tested). Determining it from supply/invoice/payment dates is a document matter (M5/M6). Tests: tests/platform/vat.test.ts, tests/unit/vat-math.test.ts M5a: Sales documents carry issue date, supply date and tax point (explicit or the issue date); the view flags taxPointReview when they differ; statutory derivation not automated (DEC-028).</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
@@ -6272,7 +6300,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts</t>
+          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6.</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
@@ -6351,9 +6379,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -6378,7 +6406,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>The snapshot function (name, kind, VAT number, account code, primary address, capture time) is delivered and tested; storing it on documents and proving history survives an edit after issue needs documents (M5/M6). Tests: tests/api/contact-roles.test.ts</t>
+          <t>The snapshot (name, kind, VAT number, account code, primary address, capture time) is stored on each sales document at approval and is proven unchanged after a later edit of the contact. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr"/>
@@ -6735,7 +6763,7 @@
         <v>25</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -6751,7 +6779,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PLANNED - specification after M3/M4 design</t>
+          <t>M5a VERIFIED (e698562; v1-m5a-acceptance.md): invoices, credit notes, allocation with realised FX, reconciliation; M5b receipts specified; M5c (VAT on foreign-currency documents) to be specified (DEC-031)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -6778,7 +6806,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -7033,7 +7061,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -7043,7 +7071,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -7053,7 +7081,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -7094,7 +7122,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6fb1938</t>
+          <t>e698562</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7134,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38311897860</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38318917124</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7195,6 +7223,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v2.6 (2026-10-12, DEC-026..031): M5a sales documents implemented. V1-MOD-06, V1-EX-01, V1-CON-04 -&gt; Implemented; V1-MOD-04, V1-EX-05, V1-CTL-02, V1-CTL-05 -&gt; Partially implemented (receipts M5b; purchases M6; alert thresholds M8); evidence extended on V1-CON-02, V1-ARC-01, MAN-ACC-06, MAN-ACC-08, XP-07, V1-VAT-04/05/07, V1-FX-07, V1-CTL-06, V1-RPT-02. No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M5b: customer receipts - allocation at entry and later, overpayments, realised FX, reversal, statement and aged receivables (DEC-032)
- Migration 20260112000000_v1_sales_receipts: sales_receipt (posted when recorded, immutable,
  unallocated amount moved only by allocations, reversed only while unallocated), allocations
  from a credit note or a receipt, receipt journals inside the sub-ledger reversal guard.
- SalesService: recordReceipt (Dr bank or cash / Cr receivables; duplicate check), allocateReceipt,
  reverseReceipt (mirror of the posted lines at the original rate), statement, agedReceivables;
  reconciliation, open balance and role-end check include receipts.
- API: 7 routes (OpenAPI). Tests: sales-receipts platform suite, database and API additions.
- Matrix v2.7: V1-MOD-08, V1-EX-03, V1-MOD-04 -> Implemented.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -704,9 +704,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -731,12 +731,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Invoices: DRAFT (no number, no ledger effect; revisioned lines) -&gt; APPROVED (numbered without gaps from a locked sequence the database checks; customer snapshot; amounts recomputed with verified VAT rates; posted as SALES_INVOICE Dr receivables / Cr revenue / Cr output VAT; journal and document linked both ways; immutable) or DISCARDED; attachments through the evidence graph; drafts from ACCEPTED AI proposals, approval by people only; positive, negative, VAT (standard, zero, exempt; exclusive, inclusive), period-lock and correction-by-credit-note tests. 'Paid' is reached by credit notes now; by receipts in M5b. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+          <t>Invoices: DRAFT (no number, no ledger effect; revisioned lines) -&gt; APPROVED (numbered without gaps from a locked sequence the database checks; customer snapshot; amounts recomputed with verified VAT rates; posted as SALES_INVOICE Dr receivables / Cr revenue / Cr output VAT; journal and document linked both ways; immutable) or DISCARDED; attachments through the evidence graph; drafts from ACCEPTED AI proposals, approval by people only; positive, negative, VAT (standard, zero, exempt; exclusive, inclusive), period-lock and correction-by-credit-note tests. 'Paid' is reached by receipts and credit notes (M5b), with statements and aged receivables. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts Tests: tests/platform/sales-receipts.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>M5a delivered; receipts (paid by payment) are M5b (DEC-026).</t>
+          <t>M5a and M5b delivered (DEC-026, DEC-032).</t>
         </is>
       </c>
     </row>
@@ -912,9 +912,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -937,7 +937,11 @@
           <t>Direct debit integration</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Receipts post SALES_RECEIPT Dr bank or cash / Cr trade receivables when recorded; allocation to one or more invoices at entry or later; part payments; overpayments kept as unallocated credit (reducing open balance, credit-limit use and ageing); realised FX on every allocation when rates differ (gain 30.00 then loss 20.00, hand-calculated); duplicate check with reason; reversal of unallocated receipts at their own rate; database guards on immutability, allocation and reversal. Tests: tests/platform/sales-receipts.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2608,9 +2612,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2633,7 +2637,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>A receipt posts exactly Dr bank (or cash) / Cr trade receivables, in functional and foreign currency; its journal links to the receipt both ways. Tests: tests/platform/sales-receipts.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts</t>
+        </is>
+      </c>
       <c r="K41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
@@ -4527,7 +4535,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2. M5a: InvoiceCreated (`invoice.created`) and `credit_note.created` are published through the outbox on approval (tests/platform/sales.test.ts); BankImported is M7.</t>
+          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2. M5a: InvoiceCreated (`invoice.created`) and `credit_note.created` are published through the outbox on approval (tests/platform/sales.test.ts); BankImported is M7. M5b adds `sales_receipt.recorded`.</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -5228,7 +5236,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts M5a: Exercised end to end for credit-note allocations (M5a): carried amounts released by `releaseShare` (full remainder or prorated), difference posted as SALES_ALLOCATION_FX to the realised-FX account with receivables lines marked adjusts_currency; hand-calculated gain 20.00 and full-settlement 16.67 cases. Receipts and payments (M5b/M6) still to come.</t>
+          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts M5a: Exercised end to end for credit-note allocations (M5a): carried amounts released by `releaseShare` (full remainder or prorated), difference posted as SALES_ALLOCATION_FX to the realised-FX account with receivables lines marked adjusts_currency; hand-calculated gain 20.00 and full-settlement 16.67 cases. Receipts and payments (M5b/M6) still to come. M5b: receipts settle foreign invoices with realised FX on every allocation, exercised end to end (two receipts at 0.90 and 0.80 against an invoice at 0.85: +30.00 / -20.00, net 10.00 = cash 860.00 less carried 850.00; no residue). Supplier payments are M6.</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -6300,7 +6308,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6.</t>
+          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6. M5b: unallocated receipts also count as open (ending refused).</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
@@ -6779,7 +6787,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>M5a VERIFIED (e698562; v1-m5a-acceptance.md): invoices, credit notes, allocation with realised FX, reconciliation; M5b receipts specified; M5c (VAT on foreign-currency documents) to be specified (DEC-031)</t>
+          <t>M5a VERIFIED (e698562); M5b implemented (receipts, allocation, realised FX, statement, ageing; acceptance package once verified); M5c (VAT on foreign-currency documents) to be specified (DEC-031)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -6806,7 +6814,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -7061,7 +7069,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7071,7 +7079,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -7081,7 +7089,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -7122,7 +7130,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>e698562</t>
+          <t>pending</t>
         </is>
       </c>
     </row>
@@ -7134,7 +7142,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38318917124</t>
+          <t>pending</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7154,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7230,6 +7238,13 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v2.7 (2026-10-13, DEC-032): M5b receipts implemented. V1-MOD-08, V1-EX-03 -&gt; Implemented; V1-MOD-04 -&gt; Implemented (paid by receipts); evidence extended on V1-FX-07 (end to end on receipts; payments M6), V1-CON-02, XP-07. No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M5b: acceptance package; matrix v2.7 regenerated with commit and CI evidence; M6 specification and decisions DEC-033..036 recorded before code (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -6787,7 +6787,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>M5a VERIFIED (e698562); M5b implemented (receipts, allocation, realised FX, statement, ageing; acceptance package once verified); M5c (VAT on foreign-currency documents) to be specified (DEC-031)</t>
+          <t>M5a VERIFIED (e698562; v1-m5a-acceptance.md); M5b VERIFIED (376aec6; v1-m5b-acceptance.md); M5c (VAT on foreign-currency documents) to be specified (DEC-031)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>376aec6</t>
         </is>
       </c>
     </row>
@@ -7142,7 +7142,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38342847878</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V1-M6a: matrix v2.8 and as-built notes (documentation only; CI evidence follows)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -761,9 +761,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -786,8 +786,16 @@
           <t>Purchase orders, expense claims</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Bills: drafts with revisioned lines (default account from the supplier profile); approval takes an internal gapless number, stores the supplier snapshot, recomputes VAT with verified rates (input VAT and reverse charge) and posts PURCHASE_BILL Dr expense or asset / Dr input VAT / Cr trade payables; immutable after approval; duplicate check on the supplier's own number (case and spaces ignored) or same date and total, with a stored reason; separate approver; period-lock and close control; hand-calculated VAT boxes (1 25.00, 4 35.00, 7 320.33). Paying bills is M6b. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>M6a delivered; payments M6b (DEC-033).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -863,9 +871,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -888,7 +896,11 @@
           <t>Supplier refund workflow</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>A debit note credits one approved bill of the same supplier and currency (database rule), uses only the bill's VAT codes at its rate versions, mirrors the reverse-charge pair, cannot exceed the bill outstanding, is allocated on approval with realised FX (credit-normal), and is traceable from both documents. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
@@ -2563,9 +2575,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2588,7 +2600,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>An approved bill posts exactly Dr expense (net per line) / Dr input VAT / Cr trade payables (gross), with zero-rated, exempt and reverse-charge lines (equal output and input VAT), hand-calculated. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
+        </is>
+      </c>
       <c r="K40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2714,9 +2730,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2741,7 +2757,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Sales: a credit note mirrors the credited lines and VAT, linked both ways (credit note -&gt; invoice; invoice lists its credit notes) and allocated. Purchases (debit notes) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+          <t>Sales: a credit note mirrors the credited lines and VAT, linked both ways (credit note -&gt; invoice; invoice lists its credit notes) and allocated. Purchases (debit notes) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts M6a: purchase debit notes mirror the credited bill lines and VAT (reverse charge included), linked both ways and allocated. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3579,9 +3595,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3606,7 +3622,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Sales invoices: before approval, another approved invoice of the same customer with the same date, currency and total, or the same customer reference, refuses approval unless a reason is given (stored on the document and audited). Supplier bills (supplier's own number) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+          <t>Sales invoices: before approval, another approved invoice of the same customer with the same date, currency and total, or the same customer reference, refuses approval unless a reason is given (stored on the document and audited). Supplier bills (supplier's own number) are M6. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts M6a: bills are checked on the supplier's own invoice number (normalised) and on date, currency and total; override needs a reason. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
@@ -4315,7 +4331,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts M5a: Close control for draft sales documents dated in the period (acknowledgement recorded); unreconciled bank items follow in M7.</t>
+          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts M5a: Close control for draft sales documents dated in the period (acknowledgement recorded); unreconciled bank items follow in M7. M6a: the close control also counts draft purchase documents.</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -5619,7 +5635,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Output VAT (sales codes) and input VAT (purchase codes) on journal lines, with visible VAT lines on the configured accounts. Invoices and bills are documents (M5/M6), so 'on invoices/bills' is not yet possible. Tests: tests/platform/vat.test.ts, tests/api/vat.test.ts M5a: Sales invoices carry output VAT per line with the verified version at the document's tax point (M5a); purchase bills are M6.</t>
+          <t>Output VAT (sales codes) and input VAT (purchase codes) on journal lines, with visible VAT lines on the configured accounts. Invoices and bills are documents (M5/M6), so 'on invoices/bills' is not yet possible. Tests: tests/platform/vat.test.ts, tests/api/vat.test.ts M5a: Sales invoices carry output VAT per line with the verified version at the document's tax point (M5a); purchase bills are M6. M6a: purchase bills carry input VAT and reverse charge per line with verified versions; workpaper boxes hand-calculated.</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
@@ -5672,7 +5688,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>A credit note entered as a debit on a sales code reduces output VAT (tested); linkage to the original supply needs documents (M5/M6). M5a: Sales credit notes adjust VAT at the rate version the invoice used, reported at the credit note's tax point (vat_rate_point proven by the database; workpaper test); purchase debit notes are M6. Rule UNVERIFIED (DEC-029).</t>
+          <t>A credit note entered as a debit on a sales code reduces output VAT (tested); linkage to the original supply needs documents (M5/M6). M5a: Sales credit notes adjust VAT at the rate version the invoice used, reported at the credit note's tax point (vat_rate_point proven by the database; workpaper test); purchase debit notes are M6. Rule UNVERIFIED (DEC-029). M6a: debit notes adjust input VAT (and the reverse-charge pair, mirrored) at the bill's rate versions. Fix found: credits on BOTH-direction codes and reverse-charge credits posted to the wrong side before M6a; fixed and regression-tested.</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr"/>
@@ -5831,7 +5847,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>Workpaper reconciliation: movement on the VAT accounts by journal date versus VAT lines by tax point, difference listed with the entries that explain it (non-VAT postings, tax points outside the journal's period). Tests: tests/platform/vat.test.ts (hand-calculated -9.50 example), tests/api/vat.test.ts</t>
+          <t>Workpaper reconciliation: movement on the VAT accounts by journal date versus VAT lines by tax point, difference listed with the entries that explain it (non-VAT postings, tax points outside the journal's period). Tests: tests/platform/vat.test.ts (hand-calculated -9.50 example), tests/api/vat.test.ts M6a: reverse charge on bills and debit notes (the pair follows the side of the net line).</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr"/>
@@ -6308,7 +6324,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6. M5b: unallocated receipts also count as open (ending refused).</t>
+          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6. M5b: unallocated receipts also count as open (ending refused). M6a: ending a supplier role is refused while it has drafts or bills with an amount outstanding.</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
@@ -6814,7 +6830,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -6830,7 +6846,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>M6a implemented (bills and debit notes; acceptance package once verified); M6b supplier payments and M6c cash transactions specified (DEC-033..036)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6857,7 +6873,7 @@
         <v>6</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -7069,7 +7085,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
@@ -7079,7 +7095,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -7089,7 +7105,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -7130,7 +7146,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>376aec6</t>
+          <t>16c7f12</t>
         </is>
       </c>
     </row>
@@ -7142,7 +7158,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38342847878</t>
+          <t>pending</t>
         </is>
       </c>
     </row>
@@ -7169,7 +7185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7245,6 +7261,13 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v2.8 (2026-10-13, DEC-033/034): M6a purchase documents implemented. V1-MOD-07, V1-EX-02, V1-EX-05, V1-CTL-02 -&gt; Implemented; V1-MOD-05 -&gt; Partially implemented (payments M6b); evidence extended on V1-VAT-04/05/08, V1-CON-02, MAN-ACC-08, including two VAT direction fixes for credits. No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M6a: acceptance package; matrix v2.8 regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -6846,7 +6846,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>M6a implemented (bills and debit notes; acceptance package once verified); M6b supplier payments and M6c cash transactions specified (DEC-033..036)</t>
+          <t>M6a VERIFIED (16c7f12; v1-m6a-acceptance.md): bills and debit notes; M6b supplier payments and M6c cash transactions specified (DEC-033..036)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38344953160</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V1-M6b: acceptance package; matrix v2.9 regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -761,9 +761,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Bills: drafts with revisioned lines (default account from the supplier profile); approval takes an internal gapless number, stores the supplier snapshot, recomputes VAT with verified rates (input VAT and reverse charge) and posts PURCHASE_BILL Dr expense or asset / Dr input VAT / Cr trade payables; immutable after approval; duplicate check on the supplier's own number (case and spaces ignored) or same date and total, with a stored reason; separate approver; period-lock and close control; hand-calculated VAT boxes (1 25.00, 4 35.00, 7 320.33). Paying bills is M6b. Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
+          <t>Bills: drafts with revisioned lines (default account from the supplier profile); approval takes an internal gapless number, stores the supplier snapshot, recomputes VAT with verified rates (input VAT and reverse charge) and posts PURCHASE_BILL Dr expense or asset / Dr input VAT / Cr trade payables; immutable after approval; duplicate check on the supplier's own number (case and spaces ignored) or same date and total, with a stored reason; separate approver; period-lock and close control; hand-calculated VAT boxes (1 25.00, 4 35.00, 7 320.33). Bills are paid by supplier payments (M6b). Tests: tests/platform/purchases.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (purchases section)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>M6a delivered; payments M6b (DEC-033).</t>
+          <t>M6a and M6b delivered (DEC-033..035).</t>
         </is>
       </c>
     </row>
@@ -977,9 +977,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1002,7 +1002,11 @@
           <t>Payment runs and bank file export</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Supplier payments post PURCHASE_PAYMENT Dr trade payables / Cr bank or cash when recorded; allocation to one or more bills at entry or later; part payments; prepayments kept as unallocated debit; realised FX on every allocation (loss 30.00 then gain 20.00, hand-calculated, net 10.00); duplicate check with reason; a payment while the supplier's stored bank details are UNVERIFIED is flagged (audited, filterable), never blocked (DEC-035); reversal of unallocated payments at their own rate; supplier statement and aged payables. Tests: tests/platform/purchase-payments.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (payments section)</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
@@ -2681,9 +2685,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2706,7 +2710,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>A payment posts exactly Dr trade payables / Cr bank (or cash), in functional and foreign currency; linked both ways. Tests: tests/platform/purchase-payments.test.ts, tests/db/purchases.test.ts, tests/api/sales.test.ts (payments section)</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
@@ -4551,7 +4559,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2. M5a: InvoiceCreated (`invoice.created`) and `credit_note.created` are published through the outbox on approval (tests/platform/sales.test.ts); BankImported is M7. M5b adds `sales_receipt.recorded`.</t>
+          <t>transaction.posted and accounting_period.state_changed events are published through the outbox; BankImported and InvoiceCreated arrive with M4 and M2. M5a: InvoiceCreated (`invoice.created`) and `credit_note.created` are published through the outbox on approval (tests/platform/sales.test.ts); BankImported is M7. M5b adds `sales_receipt.recorded`. M6 adds `bill.approved`, `debit_note.approved` and `purchase_payment.recorded`.</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -5225,9 +5233,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -5252,7 +5260,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts M5a: Exercised end to end for credit-note allocations (M5a): carried amounts released by `releaseShare` (full remainder or prorated), difference posted as SALES_ALLOCATION_FX to the realised-FX account with receivables lines marked adjusts_currency; hand-calculated gain 20.00 and full-settlement 16.67 cases. Receipts and payments (M5b/M6) still to come. M5b: receipts settle foreign invoices with realised FX on every allocation, exercised end to end (two receipts at 0.90 and 0.80 against an invoice at 0.85: +30.00 / -20.00, net 10.00 = cash 860.00 less carried 850.00; no residue). Supplier payments are M6.</t>
+          <t>Realised FX engine `settle` delivered and unit-tested (full settlement clears the carried value exactly; partial settlements prorate with no residue; gains and losses; refusals). No posting path or endpoint until receipts and payments exist (M5/M6), so not yet exercised end to end. Tests: tests/unit/fx-math.test.ts M5a: Exercised end to end for credit-note allocations (M5a): carried amounts released by `releaseShare` (full remainder or prorated), difference posted as SALES_ALLOCATION_FX to the realised-FX account with receivables lines marked adjusts_currency; hand-calculated gain 20.00 and full-settlement 16.67 cases. Receipts and payments (M5b/M6) still to come. M5b: receipts settle foreign invoices with realised FX on every allocation, exercised end to end (two receipts at 0.90 and 0.80 against an invoice at 0.85: +30.00 / -20.00, net 10.00 = cash 860.00 less carried 850.00; no residue). Supplier payments are M6. M6b: supplier payments settle foreign bills with realised FX on every allocation (credit-normal: -30.00 / +20.00), so receipts and payments both exercise it end to end.</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -6297,9 +6305,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -6324,7 +6332,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6. M5b: unallocated receipts also count as open (ending refused). M6a: ending a supplier role is refused while it has drafts or bills with an amount outstanding.</t>
+          <t>One contact holds both roles (tested); roles are created, changed, ended (with reason, never deleted) and reactivated with audit before/after. The rule 'ending is refused while open documents exist' cannot apply until documents exist (M5/M6) and is not yet implemented. Tests: tests/api/contact-roles.test.ts, tests/db/contact-roles.test.ts M5a: Ending a customer role is now refused while it has drafts or approved sales documents with an amount outstanding (tests/api/sales.test.ts); supplier documents follow in M6. M5b: unallocated receipts also count as open (ending refused). M6a: ending a supplier role is refused while it has drafts or bills with an amount outstanding. M6b: unallocated supplier payments also count as open; ending a role is now refused for open items of either role.</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
@@ -6744,7 +6752,7 @@
         <v>11</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -6787,7 +6795,7 @@
         <v>25</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -6846,7 +6854,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>M6a VERIFIED (16c7f12; v1-m6a-acceptance.md): bills and debit notes; M6b supplier payments and M6c cash transactions specified (DEC-033..036)</t>
+          <t>M6a VERIFIED (16c7f12; v1-m6a-acceptance.md); M6b VERIFIED (a753db0; v1-m6b-acceptance.md); M6c cash transactions specified (DEC-036)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6873,7 +6881,7 @@
         <v>6</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -7085,7 +7093,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -7095,7 +7103,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -7105,7 +7113,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -7146,7 +7154,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>16c7f12</t>
+          <t>a753db0</t>
         </is>
       </c>
     </row>
@@ -7158,7 +7166,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38344953160</t>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38361606618</t>
         </is>
       </c>
     </row>
@@ -7185,7 +7193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7268,6 +7276,13 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v2.9 (2026-10-13, DEC-035): M6b supplier payments implemented. V1-MOD-09, V1-EX-04, V1-MOD-05, V1-FX-07, V1-CON-02 -&gt; Implemented; evidence extended on XP-07. No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M6c: acceptance package; matrix v3.0 regenerated with commit and CI evidence (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -6870,7 +6870,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>M6a VERIFIED (16c7f12; v1-m6a-acceptance.md); M6b VERIFIED (a753db0; v1-m6b-acceptance.md); M6c cash transactions built (DEC-036/037), acceptance package after CI</t>
+          <t>M6a VERIFIED (16c7f12; v1-m6a-acceptance.md); M6b VERIFIED (a753db0; v1-m6b-acceptance.md); M6c VERIFIED (7f4adad; v1-m6c-acceptance.md)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -7168,7 +7168,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7f4adad</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7176,7 +7180,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38798396155</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V1-M7b acceptance: CI and CodeQL evidence; matrix v3.2 regenerated with commit and CI (documentation only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -7244,7 +7244,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>b8c0e0a</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7252,7 +7256,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38811610801</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V1-M8: tests, OpenAPI, matrix v3.3, plan as-built; M7b clean-clone result (full suite running before push)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -655,9 +655,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -680,8 +680,16 @@
           <t>Supplier portal</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Supplier role on the shared contact (M4a): payment terms, default currency and default expense account; bank details AES-GCM encrypted, never in lists, logs or audit (masked only), changes need a second person's verification; both roles allowed on one contact; an ended supplier role is refused on new bills and payments (contact_role_ended). Tests: tests/api/contact-roles.test.ts, tests/platform/purchases.test.ts, tests/platform/purchase-payments.test.ts, tests/unit/architecture.test.ts</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Correction recorded in v3.3: delivered by M4a (206b14d) and used by M6, but the row had not been updated. No code change.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1360,9 +1368,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1385,8 +1393,16 @@
           <t>FRS 102/105 layouts (V2)</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Profit and loss for any range with a comparative range, from journal lines only through the versioned reporting mapping (turnover, cost of sales, gross profit, administrative expenses, other operating income, operating profit, interest, profit before tax, tax, profit for the period); each line lists its accounts with general-ledger drill parameters; reconciles to the net of income and expense accounts to the cent. Hand-calculated year: turnover 3,000.00, gross profit 2,700.00, operating profit 1,675.00, profit 1,685.00 (comparative 400.00). Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>M8 delivered (DEC-043). Statutory FRS 102/105 presentation, notes and rounding are V2.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1409,9 +1425,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1434,8 +1450,16 @@
           <t>FRS 102/105 layouts (V2)</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Balance sheet as at any date with a comparative date, from journal lines only; capital and reserves include the P&amp;L cumulated to the date, split into brought forward and year to date (financial year = the accounting period containing the date); proves net assets = capital and reserves and that the trial balance balances. Hand-calculated: net assets 3,085.00 = 1,000.00 + 400.00 + 1,685.00. Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>M8 delivered (DEC-043).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1629,9 +1653,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1656,7 +1680,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Trial balance and general ledger aggregate journal_line only (architecture: no report reads source tables). P&amp;L and balance sheet are M5. Tests: tests/platform/posting-service.test.ts, tests/api/ledger.test.ts</t>
+          <t>Statements are computed in ReportService from journal_line through the reporting mapping; an architecture test fails if reports.ts reads any source-document table or writes anything. Tests: tests/unit/architecture.test.ts, tests/platform/reports.test.ts</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3062,7 +3086,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Unmatched items with ageing and counts per bank account are available through the API (unmatched list and the unmatched-line count on every bank account). Tests: tests/platform/reconciliation.test.ts, tests/db/reconciliation.test.ts, tests/api/bank.test.ts (reconciliation section)</t>
+          <t>Unmatched items with ageing and counts per bank account are available through the API (unmatched list and the unmatched-line count on every bank account). Tests: tests/platform/reconciliation.test.ts, tests/db/reconciliation.test.ts, tests/api/bank.test.ts (reconciliation section) Alert list (M8): statement lines unmatched for longer than a threshold (default 30 days), by account. Tests: tests/platform/reports.test.ts</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -3524,9 +3548,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3549,7 +3573,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>The P&amp;L equals income less expenses from the ledger for the range, and the balance sheet proves net assets = capital and reserves with a balanced trial balance, to the cent, for the current and the comparative period; the proofs are returned with each statement. Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
+        </is>
+      </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
           <t>Trial balance in M1</t>
@@ -3577,9 +3605,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3604,7 +3632,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Report -&gt; account -&gt; journal -&gt; source reference works (trial balance rows carry drill-down parameters; ledger lines carry journal and source). Source transaction and document links arrive with each source module. Tests: tests/api/ledger.test.ts M5a: Journal -&gt; sales document drill path exists (source_id) and document -&gt; journal (journal_id); report drill-down UI is M8/M9.</t>
+          <t>Statement line -&gt; accounts (with GL drill parameters) -&gt; general ledger -&gt; journal -&gt; source transaction (one resolver per journal source: documents, receipts, payments, allocations, cash transactions, transfers, requests, revaluations, reversals) -&gt; attached documents; readers without the module permission see that a source exists but not its content. A unit test fails if a journal source lacks a resolver; the platform test drills every source type in a full set of books. Tests: tests/unit/drilldown.test.ts, tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3767,12 +3795,12 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Trial balance warns about a non-zero suspense balance (account with control kind SUSPENSE). Dashboard alert is M5. Tests: tests/platform/posting-service.test.ts</t>
+          <t>The suspense balance is an alert (HIGH) as at any date, and locking a period whose end shows a suspense balance is refused unless acknowledged with a reason (recorded). Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Trial balance warning in M1; dashboard alert in M5</t>
+          <t>The dashboard screen is M9.</t>
         </is>
       </c>
     </row>
@@ -3824,12 +3852,12 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>At posting (M6c, DEC-036/037): every posting by a person that takes cash in hand below zero on its date or any later date is refused without a reason (PostingService, re-checked by the database at commit); an overdrawn bank account is returned as balanceWarnings and recorded on the audit event. Tests: tests/platform/cash.test.ts, tests/db/cash.test.ts</t>
+          <t>At posting (M6c, DEC-036/037): every posting by a person that takes cash in hand below zero on its date or any later date is refused without a reason (PostingService, re-checked by the database at commit); an overdrawn bank account is returned as balanceWarnings and recorded on the audit event. Tests: tests/platform/cash.test.ts, tests/db/cash.test.ts Alert list (M8): negative cash in hand and overdrawn bank accounts as at a date. Tests: tests/platform/reports.test.ts</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>The dashboard and alert list for negative balances remain M8.</t>
+          <t>At posting (M6c) and in the alert list (M8: negative cash HIGH, overdrawn bank MEDIUM); the dashboard screen is M9.</t>
         </is>
       </c>
     </row>
@@ -3854,9 +3882,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3881,7 +3909,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>Closing a period is refused while draft sales documents are dated in it unless acknowledged (acknowledgeDraftDocuments, recorded on the audit event); drafts are listed by status. An age threshold and alerting (dashboard) are M8. Tests: tests/platform/sales.test.ts, tests/db/sales.test.ts, tests/api/sales.test.ts, tests/unit/sales-math.test.ts</t>
+          <t>Sales and purchase drafts older than a threshold (default 14 days) are listed in the alert list, shown only to readers of the module; closing a period with drafts dated in it is refused unless acknowledged (recorded on the audit event). Tests: tests/platform/reports.test.ts, tests/platform/sales.test.ts, tests/platform/purchases.test.ts</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4294,9 +4322,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4321,7 +4349,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Journal -&gt; source via source_type/source_id/source_reference (done); source transaction -&gt; journal is delivered per source module (M2+). M5a: Sales invoices, credit notes and allocations link to their journals and back (journal source_id; document journal_id; allocation fx_journal_id), proven by database rules.</t>
+          <t>Every journal source maps to its source transaction and back (source_id on the journal; journal_id on the record); the drill-down resolver list is tested to cover every source type. Tests: tests/unit/drilldown.test.ts, tests/platform/reports.test.ts</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -4351,9 +4379,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4376,7 +4404,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Every statement figure is drillable to accounts, ledger lines, journals, source transactions and documents (V1-RPT-02). Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
+        </is>
+      </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
           <t>Same as V1-RPT-02</t>
@@ -4404,9 +4436,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -4431,7 +4463,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Explicit period states and the transition graph are delivered and enforced; the close controls so far are 'posting stops' and 'ledger balances'. Unposted documents and unreconciled bank items are added by M2-M4. Tests: tests/platform/posting-service.test.ts, tests/db/ledger.test.ts M5a: Close control for draft sales documents dated in the period (acknowledgement recorded); unreconciled bank items follow in M7. M6a: the close control also counts draft purchase documents.</t>
+          <t>Period close checks: ledger balances; FX revaluation and due reversals; draft sales and purchase documents; bank statement lines dated in the period not fully reconciled (acknowledgeUnreconciledBank); period lock checks the suspense balance (acknowledgeSuspenseBalance). Each acknowledgement is recorded with its figures on the audit event. Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4575,9 +4607,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4600,7 +4632,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>One drill-down endpoint (GET journals/{id}/source) serves every report and journal, with one resolver per source type. Tests: tests/unit/drilldown.test.ts, tests/api/reports.test.ts</t>
+        </is>
+      </c>
       <c r="K76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
@@ -5439,9 +5475,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5466,12 +5502,12 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>Reconciliation proven: after revaluation, original balance x closing rate equals the functional carrying amount per account (tests/platform/fx.test.ts); the functional-currency trial balance balances and the FX accounts' general ledger drills to the revaluation journal and its reversal (tests/api/fx.test.ts). A dedicated FX gain/loss report and multi-currency statements belong with reporting (M8).</t>
+          <t>FX report for a range: realised (allocation journals) and unrealised (revaluations and reversals) differences by currency with their journals, each drillable; open foreign-currency monetary balances against the closing rate with the difference a revaluation would post, zero once revalued; the functional trial balance balances and the P&amp;L reconciles with FX lines included. Hand-calculated: realised gain 30.00, unrealised loss 80.00 (-20.00 receivable, -60.00 bank) reversed the next day. Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Multi-currency reporting checks repeat in M8</t>
+          <t>M8 delivered (DEC-045).</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6794,7 @@
         <v>33</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -6844,7 +6880,7 @@
         <v>11</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -6887,7 +6923,7 @@
         <v>25</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -6930,7 +6966,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -7032,7 +7068,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>M8 built (DEC-043..045): statements, drill-down, alerts, close controls, FX report; acceptance package after CI</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -7047,7 +7083,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>To be written when the milestone is specified</t>
+          <t>Plan section 12: a hand-calculated year through every sub-ledger with comparatives, reconciling to the trial balance to the cent; drill-down for every journal source; alerts raised and filtered; close and lock refused and acknowledged; the FX report against the revaluation.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -7059,7 +7095,7 @@
         <v>8</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -7185,7 +7221,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -7195,7 +7231,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -7205,7 +7241,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -7244,11 +7280,7 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>b8c0e0a</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7256,11 +7288,7 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://github.com/mianshoaiblhr/UK-Accounting-Platform/actions/runs/38811610801</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7285,7 +7313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7396,6 +7424,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>v3.3 (2026-10-15, DEC-043..045): M8 reports implemented. V1-MOD-16, V1-MOD-17, V1-ARC-02, V1-RPT-01, V1-RPT-02, MAN-ACC-06, MAN-ACC-07, XP-01, V1-CTL-05, MAN-ACC-08, V1-FX-09 -&gt; Implemented; V1-CTL-03 -&gt; Partially implemented (dashboard screen M9); evidence extended on V1-CTL-04 and V1-BANK-05. Correction: V1-MOD-03 -&gt; Implemented (delivered by M4a, row not updated then). No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M9a: OpenAPI for my-access; e2e harness points supertest at the port-4000 app; periods screen keys on calendar dates; matrix v3.5
- e2e 11/11 locally (V0 journeys 4 + M9a workspace 7) against a rebuilt web app
- my-access, openapi and permissions API tests: 487 passed
- matrix v3.5: V1-CTL-03, V1-CTL-04, V1-BANK-05 implemented; V1-DOD-01 partially

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -3063,9 +3063,9 @@
           <t>M7</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3090,14 +3090,10 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Unmatched items with ageing and counts per bank account are available through the API (unmatched list and the unmatched-line count on every bank account). Tests: tests/platform/reconciliation.test.ts, tests/db/reconciliation.test.ts, tests/api/bank.test.ts (reconciliation section) Alert list (M8): statement lines unmatched for longer than a threshold (default 30 days), by account. Tests: tests/platform/reports.test.ts</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>The dashboard screen that shows the count is M9.</t>
-        </is>
-      </c>
+          <t>Unmatched items with ageing and counts per bank account are available through the API (unmatched list and the unmatched-line count on every bank account). Tests: tests/platform/reconciliation.test.ts, tests/db/reconciliation.test.ts, tests/api/bank.test.ts (reconciliation section) Alert list (M8): statement lines unmatched for longer than a threshold (default 30 days), by account. Tests: tests/platform/reports.test.ts M9a: the dashboard shows the count of statement lines unmatched beyond the threshold (from GET alerts, visible to bank:read readers) next to the other key controls; tests/e2e/workspace.test.ts. The reconciliation screens are M9c.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3772,9 +3768,9 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3799,14 +3795,10 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>The suspense balance is an alert (HIGH) as at any date, and locking a period whose end shows a suspense balance is refused unless acknowledged with a reason (recorded). Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>The dashboard screen is M9.</t>
-        </is>
-      </c>
+          <t>The suspense balance is an alert (HIGH) as at any date, and locking a period whose end shows a suspense balance is refused unless acknowledged with a reason (recorded). Tests: tests/platform/reports.test.ts, tests/api/reports.test.ts M9a (DEC-048..050): the company dashboard shows it first, from GET alerts as the API computed it, with a drill link to the account's ledger; real-browser test tests/e2e/workspace.test.ts. Locking with a suspense balance stays refused unless acknowledged with a reason (M8); the periods screen shows the API's refusal and offers that acknowledgement.</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3829,9 +3821,9 @@
           <t>M8</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3856,14 +3848,10 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>At posting (M6c, DEC-036/037): every posting by a person that takes cash in hand below zero on its date or any later date is refused without a reason (PostingService, re-checked by the database at commit); an overdrawn bank account is returned as balanceWarnings and recorded on the audit event. Tests: tests/platform/cash.test.ts, tests/db/cash.test.ts Alert list (M8): negative cash in hand and overdrawn bank accounts as at a date. Tests: tests/platform/reports.test.ts</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>At posting (M6c) and in the alert list (M8: negative cash HIGH, overdrawn bank MEDIUM); the dashboard screen is M9.</t>
-        </is>
-      </c>
+          <t>At posting (M6c, DEC-036/037): every posting by a person that takes cash in hand below zero on its date or any later date is refused without a reason (PostingService, re-checked by the database at commit); an overdrawn bank account is returned as balanceWarnings and recorded on the audit event. Tests: tests/platform/cash.test.ts, tests/db/cash.test.ts Alert list (M8): negative cash in hand and overdrawn bank accounts as at a date. Tests: tests/platform/reports.test.ts M9a (DEC-048..050): the company dashboard shows it first, from GET alerts as the API computed it, with a drill link to the account's ledger; real-browser test tests/e2e/workspace.test.ts. (cash in hand below zero and overdrawn bank, shown together).</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4721,9 +4709,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>PARTIALLY IMPLEMENTED</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -4746,7 +4734,11 @@
           <t>Mobile portal</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>M9a: workspace screens usable in a real browser behind bookkeeping.core (dashboard, accounts, journals with drill-down, trial balance, general ledger, P&amp;L, balance sheet, periods with the close and lock controls); a my-access endpoint hides what the person may not do while the API still enforces. Tests: tests/e2e/workspace.test.ts, tests/api/my-access.test.ts. Sales, purchases (M9b), bank, cash and reconciliation (M9c) screens remain.</t>
+        </is>
+      </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
           <t>DEC-002: parallel behind feature flags</t>
@@ -6798,7 +6790,7 @@
         <v>33</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -7056,7 +7048,7 @@
         <v>15</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -7099,7 +7091,7 @@
         <v>8</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -7225,7 +7217,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -7235,7 +7227,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -7245,7 +7237,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -7317,7 +7309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7442,6 +7434,13 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>v3.5 (2026-10-15, DEC-048..050, M9a): V1-CTL-03, V1-CTL-04, V1-BANK-05 -&gt; Implemented (the dashboard criterion met by the M9a workspace, real-browser tested); V1-DOD-01 Missing -&gt; Partially implemented (M9a screens; M9b and M9c remain). No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M8h and V1-M9a verified: CI 38822337045 green on 34c2c1e; acceptance packages complete; plan and matrix v3.5 regenerated with commit and CI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>M8 built (DEC-043..045): statements, drill-down, alerts, close controls, FX report; acceptance package after CI</t>
+          <t>M8 verified (code baseline b1e69af; v1-m8-acceptance.md); M8h hygiene verified (e358a26; v1-m8h-acceptance.md)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>PLANNED - runs in parallel from M2</t>
+          <t>M9a verified (34c2c1e; v1-m9a-acceptance.md): workspace screens behind bookkeeping.core; M9b sales and purchases, M9c bank, cash and reconciliation to follow</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -7276,7 +7276,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>34c2c1e</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7284,7 +7288,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/38822337045</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
V1-M9b: acceptance package draft; matrix v3.6 (evidence on V1-DOD-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -4736,7 +4736,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>M9a: workspace screens usable in a real browser behind bookkeeping.core (dashboard, accounts, journals with drill-down, trial balance, general ledger, P&amp;L, balance sheet, periods with the close and lock controls); a my-access endpoint hides what the person may not do while the API still enforces. Tests: tests/e2e/workspace.test.ts, tests/api/my-access.test.ts. Sales, purchases (M9b), bank, cash and reconciliation (M9c) screens remain.</t>
+          <t>M9a: workspace screens usable in a real browser behind bookkeeping.core (dashboard, accounts, journals with drill-down, trial balance, general ledger, P&amp;L, balance sheet, periods with the close and lock controls); a my-access endpoint hides what the person may not do while the API still enforces. Tests: tests/e2e/workspace.test.ts, tests/api/my-access.test.ts. Sales, purchases (M9b), bank, cash and reconciliation (M9c) screens remain. M9b: sales and purchases screens (documents, new invoice and bill, approve, discard, full credit and debit notes, receipts and payments with allocation and reversal, ageing, statements) with the API's override prompts; tests/e2e/subledger.test.ts.</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -7276,11 +7276,7 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>34c2c1e</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7288,11 +7284,7 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/38822337045</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7302,7 +7294,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7449,6 +7441,13 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>v3.6 (2026-10-16, M9b): evidence added to V1-DOD-01 (sales and purchases screens); no status changes. No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V1-M9c verified (CI 38973214119 and CodeQL green on c0cad12; clean clone 1881 tests, e2e 21/21); M9 complete; matrix v3.7: V1-DOD-01 implemented
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -4709,9 +4709,9 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -4736,12 +4736,12 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>M9a: workspace screens usable in a real browser behind bookkeeping.core (dashboard, accounts, journals with drill-down, trial balance, general ledger, P&amp;L, balance sheet, periods with the close and lock controls); a my-access endpoint hides what the person may not do while the API still enforces. Tests: tests/e2e/workspace.test.ts, tests/api/my-access.test.ts. Sales, purchases (M9b), bank, cash and reconciliation (M9c) screens remain. M9b: sales and purchases screens (documents, new invoice and bill, approve, discard, full credit and debit notes, receipts and payments with allocation and reversal, ageing, statements) with the API's override prompts; tests/e2e/subledger.test.ts.</t>
+          <t>M9a: workspace screens usable in a real browser behind bookkeeping.core (dashboard, accounts, journals with drill-down, trial balance, general ledger, P&amp;L, balance sheet, periods with the close and lock controls); a my-access endpoint hides what the person may not do while the API still enforces. Tests: tests/e2e/workspace.test.ts, tests/api/my-access.test.ts. Sales, purchases (M9b), bank, cash and reconciliation (M9c) screens remain. M9b: sales and purchases screens (documents, new invoice and bill, approve, discard, full credit and debit notes, receipts and payments with allocation and reversal, ageing, statements) with the API's override prompts; tests/e2e/subledger.test.ts. M9c: bank accounts, CSV statement import through the screen, reconciliation with suggestions, matching, posting from the statement, proof and sign-off, cash transactions and transfers; tests/e2e/bank.test.ts. All three slices accepted (v1-m9a/m9b/m9c-acceptance.md).</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>DEC-002: parallel behind feature flags</t>
+          <t>Screens are functional, not designed; behind bookkeeping.core; not production-approved</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>M9a verified (34c2c1e; v1-m9a-acceptance.md): workspace screens behind bookkeeping.core; M9b sales and purchases, M9c bank, cash and reconciliation to follow</t>
+          <t>M9 verified: M9a (34c2c1e), M9b (5854a0d), M9c (c0cad12); acceptance packages v1-m9a/m9b/m9c-acceptance.md; screens behind bookkeeping.core</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -7134,7 +7134,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
@@ -7227,7 +7227,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -7276,7 +7276,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>c0cad12</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7284,7 +7288,11 @@
           <t>CI</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://github.com/mianshoaiblhr/uk-accounting-platform/actions/runs/38973214119</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7309,7 +7317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7448,6 +7456,13 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v3.7 (2026-10-16, M9c): V1-DOD-01 Partially -&gt; Implemented (every V1 module has screens: M9a workspace, M9b sales and purchases, M9c bank, cash and reconciliation; real-browser tests 21/21; CI 38973214119). No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V2-M0: V2 approved (DEC-051); standard-rule verification (DEC-052), V2-M1 framework scope (DEC-053), golden trial balances (DEC-054); ADR-62..64; V2 plan with V2-M1 specified; V2 matrix (60 rows); matrix generator takes --matrix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v1-compliance-matrix.xlsx
+++ b/docs/architecture/v1-compliance-matrix.xlsx
@@ -4517,7 +4517,7 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Reporting mappings versioned in M1; VAT rates effective-dated in M2</t>
+          <t>Decided in DEC-051: reporting maps move into the database in V2-M1; tracked from now in the V2 matrix (row MAN-ACC-09). VAT rates are already effective-dated (M4b).</t>
         </is>
       </c>
     </row>
@@ -7302,7 +7302,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -7463,6 +7463,13 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>v3.8 (2026-10-17, DEC-051): MAN-ACC-09 note: decided (reporting maps into the database in V2-M1) and carried to the V2 matrix; status unchanged (Partially). No rows added or removed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>